<commit_message>
Updated workflow to allow for parallelisation
</commit_message>
<xml_diff>
--- a/tools/model_lookup.xlsx
+++ b/tools/model_lookup.xlsx
@@ -1,15 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20394"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31884FDC-9335-4B05-98AB-BC45048502D4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="5480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="1985_1997" r:id="rId3" sheetId="1"/>
-    <sheet name="1997_2009" r:id="rId4" sheetId="2"/>
-    <sheet name="2009_2018" r:id="rId5" sheetId="3"/>
+    <sheet name="1985_1997" sheetId="1" r:id="rId1"/>
+    <sheet name="1997_2009" sheetId="2" r:id="rId2"/>
+    <sheet name="2009_2018" sheetId="3" r:id="rId3"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -2917,11 +2925,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2933,7 +2940,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="darkGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
@@ -2951,15 +2958,326 @@
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I166"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="8" max="8" width="23.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2988,7 +3306,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3017,7 +3335,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -3046,7 +3364,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -3075,7 +3393,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -3104,7 +3422,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -3133,7 +3451,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -3162,7 +3480,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -3191,7 +3509,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3220,7 +3538,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -3249,7 +3567,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -3278,7 +3596,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -3307,7 +3625,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -3336,7 +3654,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -3365,7 +3683,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -3394,7 +3712,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -3423,7 +3741,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -3452,7 +3770,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -3481,7 +3799,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -3510,7 +3828,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -3539,7 +3857,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -3568,7 +3886,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -3597,7 +3915,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -3626,7 +3944,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -3655,7 +3973,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -3684,7 +4002,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -3713,7 +4031,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -3742,7 +4060,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -3771,7 +4089,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -3800,7 +4118,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -3829,7 +4147,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -3858,7 +4176,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>11</v>
       </c>
@@ -3887,7 +4205,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -3916,7 +4234,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>14</v>
       </c>
@@ -3945,7 +4263,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>15</v>
       </c>
@@ -3974,7 +4292,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>16</v>
       </c>
@@ -4003,7 +4321,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>17</v>
       </c>
@@ -4032,7 +4350,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>18</v>
       </c>
@@ -4061,7 +4379,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>19</v>
       </c>
@@ -4090,7 +4408,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>20</v>
       </c>
@@ -4119,7 +4437,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>21</v>
       </c>
@@ -4148,7 +4466,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -4177,7 +4495,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>23</v>
       </c>
@@ -4206,7 +4524,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>24</v>
       </c>
@@ -4235,7 +4553,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>25</v>
       </c>
@@ -4264,7 +4582,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>26</v>
       </c>
@@ -4293,7 +4611,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>27</v>
       </c>
@@ -4322,7 +4640,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>28</v>
       </c>
@@ -4351,7 +4669,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>29</v>
       </c>
@@ -4380,7 +4698,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -4409,7 +4727,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>31</v>
       </c>
@@ -4438,7 +4756,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>32</v>
       </c>
@@ -4467,7 +4785,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>33</v>
       </c>
@@ -4496,7 +4814,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>34</v>
       </c>
@@ -4525,7 +4843,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>35</v>
       </c>
@@ -4554,7 +4872,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>36</v>
       </c>
@@ -4583,7 +4901,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>9</v>
       </c>
@@ -4612,7 +4930,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>10</v>
       </c>
@@ -4641,7 +4959,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>11</v>
       </c>
@@ -4670,7 +4988,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>12</v>
       </c>
@@ -4699,7 +5017,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -4728,7 +5046,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>14</v>
       </c>
@@ -4757,7 +5075,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>15</v>
       </c>
@@ -4786,7 +5104,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>16</v>
       </c>
@@ -4815,7 +5133,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>17</v>
       </c>
@@ -4844,7 +5162,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>18</v>
       </c>
@@ -4873,7 +5191,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>19</v>
       </c>
@@ -4902,7 +5220,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>20</v>
       </c>
@@ -4931,7 +5249,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>21</v>
       </c>
@@ -4960,7 +5278,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>22</v>
       </c>
@@ -4989,7 +5307,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>23</v>
       </c>
@@ -5018,7 +5336,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>24</v>
       </c>
@@ -5047,7 +5365,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>25</v>
       </c>
@@ -5076,7 +5394,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>26</v>
       </c>
@@ -5105,7 +5423,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>27</v>
       </c>
@@ -5134,7 +5452,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>28</v>
       </c>
@@ -5163,7 +5481,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>29</v>
       </c>
@@ -5192,7 +5510,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>30</v>
       </c>
@@ -5221,7 +5539,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>31</v>
       </c>
@@ -5250,7 +5568,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>32</v>
       </c>
@@ -5279,7 +5597,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>33</v>
       </c>
@@ -5308,7 +5626,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>34</v>
       </c>
@@ -5337,7 +5655,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>35</v>
       </c>
@@ -5366,7 +5684,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>36</v>
       </c>
@@ -5395,7 +5713,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>9</v>
       </c>
@@ -5424,7 +5742,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>10</v>
       </c>
@@ -5453,7 +5771,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>12</v>
       </c>
@@ -5482,7 +5800,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>14</v>
       </c>
@@ -5511,7 +5829,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>15</v>
       </c>
@@ -5540,7 +5858,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>16</v>
       </c>
@@ -5569,7 +5887,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>17</v>
       </c>
@@ -5598,7 +5916,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>18</v>
       </c>
@@ -5627,7 +5945,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>19</v>
       </c>
@@ -5656,7 +5974,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>20</v>
       </c>
@@ -5685,7 +6003,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>21</v>
       </c>
@@ -5714,7 +6032,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>22</v>
       </c>
@@ -5743,7 +6061,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>23</v>
       </c>
@@ -5772,7 +6090,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>24</v>
       </c>
@@ -5801,7 +6119,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>25</v>
       </c>
@@ -5830,7 +6148,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>26</v>
       </c>
@@ -5859,7 +6177,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>27</v>
       </c>
@@ -5888,7 +6206,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>28</v>
       </c>
@@ -5917,7 +6235,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>29</v>
       </c>
@@ -5946,7 +6264,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>30</v>
       </c>
@@ -5975,7 +6293,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>31</v>
       </c>
@@ -6004,7 +6322,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>32</v>
       </c>
@@ -6033,7 +6351,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>33</v>
       </c>
@@ -6062,7 +6380,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>34</v>
       </c>
@@ -6091,7 +6409,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>35</v>
       </c>
@@ -6120,7 +6438,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>36</v>
       </c>
@@ -6149,7 +6467,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>9</v>
       </c>
@@ -6178,7 +6496,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>10</v>
       </c>
@@ -6207,7 +6525,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>11</v>
       </c>
@@ -6236,7 +6554,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>12</v>
       </c>
@@ -6265,7 +6583,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>13</v>
       </c>
@@ -6294,7 +6612,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>14</v>
       </c>
@@ -6323,7 +6641,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>15</v>
       </c>
@@ -6352,7 +6670,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>16</v>
       </c>
@@ -6381,7 +6699,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>17</v>
       </c>
@@ -6410,7 +6728,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>18</v>
       </c>
@@ -6439,7 +6757,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>19</v>
       </c>
@@ -6468,7 +6786,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>20</v>
       </c>
@@ -6497,7 +6815,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>21</v>
       </c>
@@ -6526,7 +6844,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>22</v>
       </c>
@@ -6555,7 +6873,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>23</v>
       </c>
@@ -6584,7 +6902,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>24</v>
       </c>
@@ -6613,7 +6931,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>25</v>
       </c>
@@ -6642,7 +6960,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>26</v>
       </c>
@@ -6671,7 +6989,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>27</v>
       </c>
@@ -6700,7 +7018,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>28</v>
       </c>
@@ -6729,7 +7047,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>29</v>
       </c>
@@ -6758,7 +7076,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>30</v>
       </c>
@@ -6787,7 +7105,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>31</v>
       </c>
@@ -6816,7 +7134,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>32</v>
       </c>
@@ -6845,7 +7163,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>33</v>
       </c>
@@ -6874,7 +7192,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>34</v>
       </c>
@@ -6903,7 +7221,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>35</v>
       </c>
@@ -6932,7 +7250,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>36</v>
       </c>
@@ -6961,7 +7279,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="139">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>9</v>
       </c>
@@ -6990,7 +7308,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>10</v>
       </c>
@@ -7019,7 +7337,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>11</v>
       </c>
@@ -7048,7 +7366,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>12</v>
       </c>
@@ -7077,7 +7395,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>13</v>
       </c>
@@ -7106,7 +7424,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>14</v>
       </c>
@@ -7135,7 +7453,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>15</v>
       </c>
@@ -7164,7 +7482,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>16</v>
       </c>
@@ -7193,7 +7511,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>17</v>
       </c>
@@ -7222,7 +7540,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>18</v>
       </c>
@@ -7251,7 +7569,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>19</v>
       </c>
@@ -7280,7 +7598,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>20</v>
       </c>
@@ -7309,7 +7627,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>21</v>
       </c>
@@ -7338,7 +7656,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>22</v>
       </c>
@@ -7367,7 +7685,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="153">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>23</v>
       </c>
@@ -7396,7 +7714,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="154">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>24</v>
       </c>
@@ -7425,7 +7743,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="155">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>25</v>
       </c>
@@ -7454,7 +7772,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="156">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>26</v>
       </c>
@@ -7483,7 +7801,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="157">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>27</v>
       </c>
@@ -7512,7 +7830,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="158">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>28</v>
       </c>
@@ -7541,7 +7859,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>29</v>
       </c>
@@ -7570,7 +7888,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>30</v>
       </c>
@@ -7599,7 +7917,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>31</v>
       </c>
@@ -7628,7 +7946,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="162">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>32</v>
       </c>
@@ -7657,7 +7975,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="163">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>33</v>
       </c>
@@ -7686,7 +8004,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>34</v>
       </c>
@@ -7715,7 +8033,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="165">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>35</v>
       </c>
@@ -7744,7 +8062,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="166">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>36</v>
       </c>
@@ -7774,16 +8092,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:I154"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7812,7 +8130,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -7841,7 +8159,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -7870,7 +8188,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -7899,7 +8217,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -7928,7 +8246,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -7957,7 +8275,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -7986,7 +8304,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -8015,7 +8333,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -8044,7 +8362,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -8073,7 +8391,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -8102,7 +8420,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -8131,7 +8449,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -8160,7 +8478,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -8189,7 +8507,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -8218,7 +8536,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -8247,7 +8565,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -8276,7 +8594,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -8305,7 +8623,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -8334,7 +8652,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -8363,7 +8681,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -8392,7 +8710,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -8421,7 +8739,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>413</v>
       </c>
@@ -8450,7 +8768,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -8479,7 +8797,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -8508,7 +8826,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -8537,7 +8855,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -8566,7 +8884,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>10</v>
       </c>
@@ -8595,7 +8913,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -8624,7 +8942,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -8653,7 +8971,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>14</v>
       </c>
@@ -8682,7 +9000,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -8711,7 +9029,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>17</v>
       </c>
@@ -8740,7 +9058,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>18</v>
       </c>
@@ -8769,7 +9087,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>19</v>
       </c>
@@ -8798,7 +9116,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -8827,7 +9145,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -8856,7 +9174,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>22</v>
       </c>
@@ -8885,7 +9203,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>23</v>
       </c>
@@ -8914,7 +9232,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>24</v>
       </c>
@@ -8943,7 +9261,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>25</v>
       </c>
@@ -8972,7 +9290,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>26</v>
       </c>
@@ -9001,7 +9319,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>27</v>
       </c>
@@ -9030,7 +9348,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -9059,7 +9377,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>29</v>
       </c>
@@ -9088,7 +9406,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>30</v>
       </c>
@@ -9117,7 +9435,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>32</v>
       </c>
@@ -9146,7 +9464,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>413</v>
       </c>
@@ -9175,7 +9493,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>33</v>
       </c>
@@ -9204,7 +9522,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>34</v>
       </c>
@@ -9233,7 +9551,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -9262,7 +9580,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>36</v>
       </c>
@@ -9291,7 +9609,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>10</v>
       </c>
@@ -9320,7 +9638,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>11</v>
       </c>
@@ -9349,7 +9667,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>12</v>
       </c>
@@ -9378,7 +9696,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -9407,7 +9725,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -9436,7 +9754,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>15</v>
       </c>
@@ -9465,7 +9783,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>17</v>
       </c>
@@ -9494,7 +9812,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>18</v>
       </c>
@@ -9523,7 +9841,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>19</v>
       </c>
@@ -9552,7 +9870,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>20</v>
       </c>
@@ -9581,7 +9899,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>21</v>
       </c>
@@ -9610,7 +9928,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>22</v>
       </c>
@@ -9639,7 +9957,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>23</v>
       </c>
@@ -9668,7 +9986,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>24</v>
       </c>
@@ -9697,7 +10015,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>25</v>
       </c>
@@ -9726,7 +10044,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>26</v>
       </c>
@@ -9755,7 +10073,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>27</v>
       </c>
@@ -9784,7 +10102,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>28</v>
       </c>
@@ -9813,7 +10131,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>29</v>
       </c>
@@ -9842,7 +10160,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>30</v>
       </c>
@@ -9871,7 +10189,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>32</v>
       </c>
@@ -9900,7 +10218,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>413</v>
       </c>
@@ -9929,7 +10247,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>33</v>
       </c>
@@ -9958,7 +10276,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>34</v>
       </c>
@@ -9987,7 +10305,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>35</v>
       </c>
@@ -10016,7 +10334,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>36</v>
       </c>
@@ -10045,7 +10363,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>10</v>
       </c>
@@ -10074,7 +10392,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -10103,7 +10421,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>12</v>
       </c>
@@ -10132,7 +10450,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>14</v>
       </c>
@@ -10161,7 +10479,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>15</v>
       </c>
@@ -10190,7 +10508,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>17</v>
       </c>
@@ -10219,7 +10537,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>18</v>
       </c>
@@ -10248,7 +10566,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>19</v>
       </c>
@@ -10277,7 +10595,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>20</v>
       </c>
@@ -10306,7 +10624,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -10335,7 +10653,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -10364,7 +10682,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>23</v>
       </c>
@@ -10393,7 +10711,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>24</v>
       </c>
@@ -10422,7 +10740,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>25</v>
       </c>
@@ -10451,7 +10769,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>26</v>
       </c>
@@ -10480,7 +10798,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>27</v>
       </c>
@@ -10509,7 +10827,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>28</v>
       </c>
@@ -10538,7 +10856,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>29</v>
       </c>
@@ -10567,7 +10885,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>30</v>
       </c>
@@ -10596,7 +10914,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>32</v>
       </c>
@@ -10625,7 +10943,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>33</v>
       </c>
@@ -10654,7 +10972,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>34</v>
       </c>
@@ -10683,7 +11001,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>35</v>
       </c>
@@ -10712,7 +11030,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>36</v>
       </c>
@@ -10741,7 +11059,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>10</v>
       </c>
@@ -10770,7 +11088,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>11</v>
       </c>
@@ -10799,7 +11117,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>12</v>
       </c>
@@ -10828,7 +11146,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>13</v>
       </c>
@@ -10857,7 +11175,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>14</v>
       </c>
@@ -10886,7 +11204,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>15</v>
       </c>
@@ -10915,7 +11233,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>17</v>
       </c>
@@ -10944,7 +11262,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>18</v>
       </c>
@@ -10973,7 +11291,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>19</v>
       </c>
@@ -11002,7 +11320,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>20</v>
       </c>
@@ -11031,7 +11349,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>21</v>
       </c>
@@ -11060,7 +11378,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>22</v>
       </c>
@@ -11089,7 +11407,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>23</v>
       </c>
@@ -11118,7 +11436,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>24</v>
       </c>
@@ -11147,7 +11465,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>25</v>
       </c>
@@ -11176,7 +11494,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>26</v>
       </c>
@@ -11205,7 +11523,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>27</v>
       </c>
@@ -11234,7 +11552,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>28</v>
       </c>
@@ -11263,7 +11581,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>29</v>
       </c>
@@ -11292,7 +11610,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>30</v>
       </c>
@@ -11321,7 +11639,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>32</v>
       </c>
@@ -11350,7 +11668,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>413</v>
       </c>
@@ -11379,7 +11697,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>33</v>
       </c>
@@ -11408,7 +11726,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>34</v>
       </c>
@@ -11437,7 +11755,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>35</v>
       </c>
@@ -11466,7 +11784,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>36</v>
       </c>
@@ -11495,7 +11813,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>10</v>
       </c>
@@ -11524,7 +11842,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>11</v>
       </c>
@@ -11553,7 +11871,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>12</v>
       </c>
@@ -11582,7 +11900,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>13</v>
       </c>
@@ -11611,7 +11929,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>14</v>
       </c>
@@ -11640,7 +11958,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>15</v>
       </c>
@@ -11669,7 +11987,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>17</v>
       </c>
@@ -11698,7 +12016,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>18</v>
       </c>
@@ -11727,7 +12045,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>19</v>
       </c>
@@ -11756,7 +12074,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>20</v>
       </c>
@@ -11785,7 +12103,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="139">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>21</v>
       </c>
@@ -11814,7 +12132,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>22</v>
       </c>
@@ -11843,7 +12161,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>23</v>
       </c>
@@ -11872,7 +12190,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>24</v>
       </c>
@@ -11901,7 +12219,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>25</v>
       </c>
@@ -11930,7 +12248,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>26</v>
       </c>
@@ -11959,7 +12277,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>27</v>
       </c>
@@ -11988,7 +12306,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>28</v>
       </c>
@@ -12017,7 +12335,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>29</v>
       </c>
@@ -12046,7 +12364,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>30</v>
       </c>
@@ -12075,7 +12393,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>32</v>
       </c>
@@ -12104,7 +12422,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>413</v>
       </c>
@@ -12133,7 +12451,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>33</v>
       </c>
@@ -12162,7 +12480,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>34</v>
       </c>
@@ -12191,7 +12509,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="153">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>35</v>
       </c>
@@ -12220,7 +12538,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="154">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>36</v>
       </c>
@@ -12250,16 +12568,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:I123"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12288,7 +12606,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -12317,7 +12635,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -12346,7 +12664,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -12375,7 +12693,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -12404,7 +12722,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -12433,7 +12751,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -12462,7 +12780,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -12491,7 +12809,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -12520,7 +12838,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -12549,7 +12867,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -12578,7 +12896,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -12607,7 +12925,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -12636,7 +12954,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -12665,7 +12983,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -12694,7 +13012,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -12723,7 +13041,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -12752,7 +13070,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -12781,7 +13099,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>413</v>
       </c>
@@ -12810,7 +13128,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -12839,7 +13157,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -12868,7 +13186,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -12897,7 +13215,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -12926,7 +13244,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -12955,7 +13273,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -12984,7 +13302,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -13013,7 +13331,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -13042,7 +13360,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>16</v>
       </c>
@@ -13071,7 +13389,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -13100,7 +13418,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>19</v>
       </c>
@@ -13129,7 +13447,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -13158,7 +13476,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -13187,7 +13505,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -13216,7 +13534,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>24</v>
       </c>
@@ -13245,7 +13563,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>25</v>
       </c>
@@ -13274,7 +13592,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -13303,7 +13621,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>30</v>
       </c>
@@ -13332,7 +13650,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>32</v>
       </c>
@@ -13361,7 +13679,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>413</v>
       </c>
@@ -13390,7 +13708,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>33</v>
       </c>
@@ -13419,7 +13737,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>34</v>
       </c>
@@ -13448,7 +13766,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>36</v>
       </c>
@@ -13477,7 +13795,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>10</v>
       </c>
@@ -13506,7 +13824,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -13535,7 +13853,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>12</v>
       </c>
@@ -13564,7 +13882,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -13593,7 +13911,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>14</v>
       </c>
@@ -13622,7 +13940,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -13651,7 +13969,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -13680,7 +13998,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>18</v>
       </c>
@@ -13709,7 +14027,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>19</v>
       </c>
@@ -13738,7 +14056,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>20</v>
       </c>
@@ -13767,7 +14085,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>22</v>
       </c>
@@ -13796,7 +14114,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>23</v>
       </c>
@@ -13825,7 +14143,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>24</v>
       </c>
@@ -13854,7 +14172,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>25</v>
       </c>
@@ -13883,7 +14201,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>29</v>
       </c>
@@ -13912,7 +14230,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>30</v>
       </c>
@@ -13941,7 +14259,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>32</v>
       </c>
@@ -13970,7 +14288,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>413</v>
       </c>
@@ -13999,7 +14317,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>33</v>
       </c>
@@ -14028,7 +14346,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>34</v>
       </c>
@@ -14057,7 +14375,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>36</v>
       </c>
@@ -14086,7 +14404,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>10</v>
       </c>
@@ -14115,7 +14433,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>12</v>
       </c>
@@ -14144,7 +14462,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>14</v>
       </c>
@@ -14173,7 +14491,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>15</v>
       </c>
@@ -14202,7 +14520,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>16</v>
       </c>
@@ -14231,7 +14549,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>18</v>
       </c>
@@ -14260,7 +14578,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>19</v>
       </c>
@@ -14289,7 +14607,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>20</v>
       </c>
@@ -14318,7 +14636,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>22</v>
       </c>
@@ -14347,7 +14665,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>23</v>
       </c>
@@ -14376,7 +14694,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>24</v>
       </c>
@@ -14405,7 +14723,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>25</v>
       </c>
@@ -14434,7 +14752,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>29</v>
       </c>
@@ -14463,7 +14781,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>30</v>
       </c>
@@ -14492,7 +14810,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>32</v>
       </c>
@@ -14521,7 +14839,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>33</v>
       </c>
@@ -14550,7 +14868,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>34</v>
       </c>
@@ -14579,7 +14897,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>36</v>
       </c>
@@ -14608,7 +14926,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>10</v>
       </c>
@@ -14637,7 +14955,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>11</v>
       </c>
@@ -14666,7 +14984,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>12</v>
       </c>
@@ -14695,7 +15013,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>13</v>
       </c>
@@ -14724,7 +15042,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>14</v>
       </c>
@@ -14753,7 +15071,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>15</v>
       </c>
@@ -14782,7 +15100,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>16</v>
       </c>
@@ -14811,7 +15129,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>18</v>
       </c>
@@ -14840,7 +15158,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>19</v>
       </c>
@@ -14869,7 +15187,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>20</v>
       </c>
@@ -14898,7 +15216,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>22</v>
       </c>
@@ -14927,7 +15245,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>23</v>
       </c>
@@ -14956,7 +15274,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>24</v>
       </c>
@@ -14985,7 +15303,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>25</v>
       </c>
@@ -15014,7 +15332,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>29</v>
       </c>
@@ -15043,7 +15361,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>30</v>
       </c>
@@ -15072,7 +15390,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>32</v>
       </c>
@@ -15101,7 +15419,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>413</v>
       </c>
@@ -15130,7 +15448,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>33</v>
       </c>
@@ -15159,7 +15477,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>34</v>
       </c>
@@ -15188,7 +15506,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>36</v>
       </c>
@@ -15217,7 +15535,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>10</v>
       </c>
@@ -15246,7 +15564,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>11</v>
       </c>
@@ -15275,7 +15593,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>12</v>
       </c>
@@ -15304,7 +15622,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>13</v>
       </c>
@@ -15333,7 +15651,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>14</v>
       </c>
@@ -15362,7 +15680,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>15</v>
       </c>
@@ -15391,7 +15709,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>16</v>
       </c>
@@ -15420,7 +15738,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>18</v>
       </c>
@@ -15449,7 +15767,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>19</v>
       </c>
@@ -15478,7 +15796,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>20</v>
       </c>
@@ -15507,7 +15825,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>22</v>
       </c>
@@ -15536,7 +15854,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>23</v>
       </c>
@@ -15565,7 +15883,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>24</v>
       </c>
@@ -15594,7 +15912,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>25</v>
       </c>
@@ -15623,7 +15941,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>29</v>
       </c>
@@ -15652,7 +15970,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>30</v>
       </c>
@@ -15681,7 +15999,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>32</v>
       </c>
@@ -15710,7 +16028,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>413</v>
       </c>
@@ -15739,7 +16057,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>33</v>
       </c>
@@ -15768,7 +16086,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>34</v>
       </c>
@@ -15797,7 +16115,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>36</v>
       </c>
@@ -15827,6 +16145,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>